<commit_message>
feat: Enhance product import functionality and stock management
- Added informative messages in the ImportProducts component regarding product updates and stock handling.
- Updated StockEntryForm to include currentBranchId for better stock tracking.
- Modified Product interface to include branch_stock for accurate stock representation.
- Introduced a new API endpoint for fetching stock by product IDs.
- Secured product import and export routes with authentication middleware.
- Implemented tests for product import functionality, ensuring correct stock updates and handling of invalid quantities.
- Created NoteStockService to manage stock adjustments related to notes, including handling cancellations and restorations.
- Added comprehensive tests for note stock management, ensuring correct stock behavior during note creation, editing, and deletion.
- Developed e2e tests for product import and stock warnings, ensuring user experience aligns with stock availability.
</commit_message>
<xml_diff>
--- a/public/templates/template_productos.xlsx
+++ b/public/templates/template_productos.xlsx
@@ -1,39 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10209"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jovannyramirez/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A77E5099-F83B-F545-93F6-EF2E52237E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" forceFullCalc="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>MARCA</t>
   </si>
@@ -72,30 +54,43 @@
   </si>
   <si>
     <t>PIEZA</t>
+  </si>
+  <si>
+    <t>EXISTENCIAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <b/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -125,23 +120,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -431,22 +418,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="8.83203125" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="0"/>
+    <col min="2" max="2" width="26.83203125" customWidth="true" style="0"/>
+    <col min="3" max="3" width="10.33203125" customWidth="true" style="0"/>
+    <col min="4" max="4" width="5.6640625" customWidth="true" style="0"/>
+    <col min="5" max="5" width="10.33203125" customWidth="true" style="0"/>
+    <col min="6" max="6" width="22.33203125" customWidth="true" style="0"/>
+    <col min="7" max="7" width="8.83203125" style="0"/>
+    <col min="8" max="8" width="5.6640625" customWidth="true" style="0"/>
+    <col min="9" max="9" width="8.83203125" style="0"/>
+    <col min="10" max="10" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" customHeight="1" ht="19">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -474,8 +465,11 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" customHeight="1" ht="19">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -503,9 +497,22 @@
       <c r="I2" s="1">
         <v>5</v>
       </c>
+      <c r="J2" s="1">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup paperSize="1" orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add test for downloadable template import with price2 validation
</commit_message>
<xml_diff>
--- a/public/templates/template_productos.xlsx
+++ b/public/templates/template_productos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>MARCA</t>
   </si>
@@ -35,28 +35,31 @@
     <t>PRECIO PUBLICO</t>
   </si>
   <si>
+    <t>APPLE</t>
+  </si>
+  <si>
+    <t>iPhone 16 PRO MAX</t>
+  </si>
+  <si>
+    <t>10x2</t>
+  </si>
+  <si>
+    <t>PIEZA</t>
+  </si>
+  <si>
+    <t>EXISTENCIAS</t>
+  </si>
+  <si>
+    <t>EXTRA</t>
+  </si>
+  <si>
+    <t>IVA</t>
+  </si>
+  <si>
     <t>COSTO</t>
   </si>
   <si>
-    <t>IVA</t>
-  </si>
-  <si>
-    <t>EXTRA</t>
-  </si>
-  <si>
-    <t>APPLE</t>
-  </si>
-  <si>
-    <t>iPhone 16 PRO MAX</t>
-  </si>
-  <si>
-    <t>10x2</t>
-  </si>
-  <si>
-    <t>PIEZA</t>
-  </si>
-  <si>
-    <t>EXISTENCIAS</t>
+    <t>PRECIO 2</t>
   </si>
 </sst>
 </file>
@@ -422,7 +425,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="8.83203125" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="0"/>
@@ -431,13 +434,14 @@
     <col min="4" max="4" width="5.6640625" customWidth="true" style="0"/>
     <col min="5" max="5" width="10.33203125" customWidth="true" style="0"/>
     <col min="6" max="6" width="22.33203125" customWidth="true" style="0"/>
-    <col min="7" max="7" width="8.83203125" style="0"/>
-    <col min="8" max="8" width="5.6640625" customWidth="true" style="0"/>
-    <col min="9" max="9" width="8.83203125" style="0"/>
-    <col min="10" max="10" width="14" customWidth="true" style="0"/>
+    <col min="7" max="7" width="22.33203125" customWidth="true" style="0"/>
+    <col min="8" max="8" width="8.83203125" style="0"/>
+    <col min="9" max="9" width="5.6640625" customWidth="true" style="0"/>
+    <col min="10" max="10" width="8.83203125" style="0"/>
+    <col min="11" max="11" width="14" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" customHeight="1" ht="19">
+    <row r="1" spans="1:11" customHeight="1" ht="19">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -457,47 +461,53 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" customHeight="1" ht="19">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" customHeight="1" ht="19">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="D2" s="1">
         <v>0.1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F2" s="1">
         <v>1300</v>
       </c>
       <c r="G2" s="1">
+        <v>1200</v>
+      </c>
+      <c r="H2" s="1">
         <v>1000</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>16</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>5</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="1">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add skip_global_extra field to products and update related logic for effective extra calculations
</commit_message>
<xml_diff>
--- a/public/templates/template_productos.xlsx
+++ b/public/templates/template_productos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>MARCA</t>
   </si>
@@ -35,6 +35,21 @@
     <t>PRECIO PUBLICO</t>
   </si>
   <si>
+    <t>PRECIO 2</t>
+  </si>
+  <si>
+    <t>COSTO</t>
+  </si>
+  <si>
+    <t>IVA</t>
+  </si>
+  <si>
+    <t>EXTRA</t>
+  </si>
+  <si>
+    <t>EXISTENCIAS</t>
+  </si>
+  <si>
     <t>APPLE</t>
   </si>
   <si>
@@ -47,19 +62,7 @@
     <t>PIEZA</t>
   </si>
   <si>
-    <t>EXISTENCIAS</t>
-  </si>
-  <si>
-    <t>EXTRA</t>
-  </si>
-  <si>
-    <t>IVA</t>
-  </si>
-  <si>
-    <t>COSTO</t>
-  </si>
-  <si>
-    <t>PRECIO 2</t>
+    <t>SIN EXTRA GLOBAL</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="8.83203125" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="0"/>
@@ -439,9 +442,10 @@
     <col min="9" max="9" width="5.6640625" customWidth="true" style="0"/>
     <col min="10" max="10" width="8.83203125" style="0"/>
     <col min="11" max="11" width="14" customWidth="true" style="0"/>
+    <col min="12" max="12" width="25.422" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" customHeight="1" ht="19">
+    <row r="1" spans="1:12" customHeight="1" ht="19">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -461,36 +465,39 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" customHeight="1" ht="19">
+    <row r="2" spans="1:12" customHeight="1" ht="19">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1">
         <v>0.1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1">
         <v>1300</v>

</xml_diff>